<commit_message>
COT-2026-0160 — el itinerario de la planilla en español y en inglés
Agrega la hoja «Itinerary», espejo exacto de «Itinerario»: mismas
columnas, mismos bloques, mismos números de servicio y las mismas dos
columnas en amarillo para que respondan. Cambian sólo los rótulos y los
nombres de día.

El contenido no se duplica: los textos de cada bloque ya venían bilingües
de itinerario.mjs, así que la hoja se arma con la misma función llamada
dos veces y las dos versiones no pueden divergir.

Las hojas Preguntas y Referencia siguen en español: la primera va para
Francisco y la segunda es interna.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CyDPBBPEqC3tR4tfkkVi9f
</commit_message>
<xml_diff>
--- a/cotizaciones/segar-san-pedro-atacama/Tourevo-COT-2026-0160-Segar-Itinerario-para-operador.xlsx
+++ b/cotizaciones/segar-san-pedro-atacama/Tourevo-COT-2026-0160-Segar-Itinerario-para-operador.xlsx
@@ -9,13 +9,16 @@
   </bookViews>
   <sheets>
     <sheet name="Itinerario" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Preguntas" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Referencia" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Itinerary" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Preguntas" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Referencia" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">Itinerario!$4:$4</definedName>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Itinerario!$A$4:$J$25</definedName>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">Preguntas!$4:$4</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">Itinerary!$4:$4</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Itinerary!$A$4:$J$25</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Titles" vbProcedure="false">Preguntas!$4:$4</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="211">
   <si>
     <t xml:space="preserve">Segar · San Pedro de Atacama · 22 al 26 de diciembre de 2026 · 4 pasajeros</t>
   </si>
@@ -299,6 +302,173 @@
   </si>
   <si>
     <t xml:space="preserve">Vuelo Santiago → Dallas · AA940</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segar · San Pedro de Atacama · 22 to 26 December 2026 · 4 travellers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FOR THE OPERATOR: fill in only columns I (“Feasible?”) and J (“Comments”), in yellow. Everything else is for reference. Under “Feasible?” put Yes, No or With changes. Column Nº numbers the 9 services we operate: rows without a number are flights, meals or free time. Rows in amber changed or need a decision.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Start</t>
+  </si>
+  <si>
+    <t xml:space="preserve">End</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operated by</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What we need confirmed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feasible?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operator comments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">example</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXAMPLE — delete this row</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is what a filled line looks like.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With changes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doable, but departure at 10:00.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tuesday 22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flight Santiago → Calama (CJC) · LATAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Client</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transfer Calama → San Pedro de Atacama
+The operator calculates the transfer at 1 h 45, not the hour we had: you reach the hotel at 20:00, not 19:15. Departure from the airport at 18:15, 35 minutes after the flight lands.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Are 35 minutes between the 17:41 landing and the transfer departure enough, or should we leave more?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arrival and check-in at the hotel · rest of the evening free</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wednesday 23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pukará de Quitor · guided
+With the 26th free and Cejar taking the afternoon, the morning of the 23rd is the only gap left for Quitor. Two gentle hours a step from the village, so it does not spoil the settling-in day.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The operator notes Quitor and the sandboarding are two separate excursions even within one half day. Here they fall on different days, so they bill separately anyway. Do you confirm 09:30 – 11:30 on the 23rd?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lunch and rest at the hotel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laguna Cejar · floating at Laguna Piedra + Ojos de Tebenquiche + Tebenquiche Lagoon
+It runs in the afternoon because agencies cannot operate Cejar in the morning. The time is the one the operator proposed. The relaxed-morning idea still holds: the 23rd starts late with only two hours of Quitor before it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmed 15:30 – 19:30 on Wednesday the 23rd?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Back to the hotel, shower and rest
+An hour and a half between leaving the salt water and heading out under the sky.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Astronomy tour · shared
+Back to the 23rd and to the shared format, which is what was quoted: CLP 40,000 per person against the CLP 600,000 for the group the private tour costs on the 24th. It is also the night Segar asked about.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the shared tour run on the night of the 23rd and does CLP 40,000 per person hold? Note: that night the moon is 99.9% illuminated — the 24th is the same, so switching nights changes nothing. Better to have the guide aim it at the moon and planets.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thursday 24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puritama Hot Springs · 3,500 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is there a Christmas Eve supplement on Puritama? And is it feasible to be back in San Pedro by 13:30, with the next departure at 14:30?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lunch and rest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valle de la Muerte · sandboarding
+This is what has already been confirmed to Segar for the 24th. It chains into Valle de la Luna, which sits right next door, with half an hour in between.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can you chain sandboarding 14:30 – 16:30 into Vallecito 17:00 – 21:00 on the same day, with half an hour between? They are in the same area, but the operator asked for buffer and we want it to hold.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valle de la Luna South · Vallecito at sunset
+It leaves at 17:00 because the operator warns that at 17:30 there is no longer time to do it properly. And it moves to the 24th because Cejar takes the 23rd: both are afternoon excursions and cannot share a day.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmed 17:00 – 21:00 on the 24th? Is there a Christmas Eve supplement?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Christmas Eve dinner
+Segar has to confirm this. It was at 20:00, but Vallecito ends at 21:00. Either dinner moves to 21:30 — which for Christmas Eve in Chile is the normal hour — or Valle de la Luna cannot go on the 24th. No transfer from us: they take the hotel shuttle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Friday 25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Altiplano · Laguna Chaxa, Toconao, Miscanti and Piedras Rojas
+With Chaxa in, the operator runs it 08:00 to 18:00 and the 25 December rate lands at CLP 270,000 per person, against the 210,000 quoted. They tell us they do not recommend it: it makes for a very long day. Drop Chaxa and it gets shorter and cheaper.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How much is the Chaxa entrance fee, to add it to the ones bought in advance? And if Chaxa comes out, what do the price and timing become?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dinner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saturday 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free morning in San Pedro · breakfast and check-out
+The last day carries no excursions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transfer San Pedro → Calama
+Brought forward to 10:00: at 1 h 45 for the transfer, leaving at 10:24 gave under two hours before the flight. It arrives 11:45 for the 13:44 flight.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you confirm 10:00 hotel pickup to reach Calama at 11:45?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flight Calama → Santiago · LATAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">International check-in in Santiago</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flight Santiago → Dallas · AA940</t>
   </si>
   <si>
     <t xml:space="preserve">Preguntas que no cuelgan de una línea del itinerario</t>
@@ -992,6 +1162,10 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
@@ -1817,6 +1991,648 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
+  <dimension ref="A1:J25"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="40"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5"/>
+      <c r="B6" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="H6" s="6"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+    </row>
+    <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="I7" s="13"/>
+      <c r="J7" s="13"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5"/>
+      <c r="B8" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="H8" s="6"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+    </row>
+    <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="I9" s="13"/>
+      <c r="J9" s="13"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5"/>
+      <c r="B10" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="H10" s="6"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+    </row>
+    <row r="11" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="I11" s="13"/>
+      <c r="J11" s="13"/>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5"/>
+      <c r="B12" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="H12" s="6"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+    </row>
+    <row r="13" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="I13" s="13"/>
+      <c r="J13" s="13"/>
+    </row>
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>120</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="I14" s="13"/>
+      <c r="J14" s="13"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5"/>
+      <c r="B15" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="H15" s="6"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+    </row>
+    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="G16" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="H16" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="I16" s="13"/>
+      <c r="J16" s="13"/>
+    </row>
+    <row r="17" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="I17" s="13"/>
+      <c r="J17" s="13"/>
+    </row>
+    <row r="18" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="17"/>
+      <c r="B18" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="E18" s="19"/>
+      <c r="F18" s="18" t="s">
+        <v>127</v>
+      </c>
+      <c r="G18" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="H18" s="18"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+    </row>
+    <row r="19" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="F19" s="16" t="s">
+        <v>129</v>
+      </c>
+      <c r="G19" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="H19" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="I19" s="13"/>
+      <c r="J19" s="13"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5"/>
+      <c r="B20" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="H20" s="6"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5"/>
+      <c r="B21" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="H21" s="6"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
+    </row>
+    <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="D22" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="G22" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H22" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="I22" s="13"/>
+      <c r="J22" s="13"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5"/>
+      <c r="B23" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="H23" s="6"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5"/>
+      <c r="B24" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="H24" s="6"/>
+      <c r="I24" s="8"/>
+      <c r="J24" s="8"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5"/>
+      <c r="B25" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="H25" s="6"/>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:J25"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -1828,12 +2644,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="20" t="s">
-        <v>87</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="21" t="s">
-        <v>88</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1841,13 +2657,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>89</v>
+        <v>141</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1861,7 +2677,7 @@
         <v>18</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>92</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1869,10 +2685,10 @@
         <v>1</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>93</v>
+        <v>145</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>94</v>
+        <v>146</v>
       </c>
       <c r="D6" s="13"/>
     </row>
@@ -1881,10 +2697,10 @@
         <v>2</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>95</v>
+        <v>147</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>96</v>
+        <v>148</v>
       </c>
       <c r="D7" s="13"/>
     </row>
@@ -1893,10 +2709,10 @@
         <v>3</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>97</v>
+        <v>149</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>98</v>
+        <v>150</v>
       </c>
       <c r="D8" s="13"/>
     </row>
@@ -1905,10 +2721,10 @@
         <v>4</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>99</v>
+        <v>151</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>100</v>
+        <v>152</v>
       </c>
       <c r="D9" s="13"/>
     </row>
@@ -1923,7 +2739,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -1939,12 +2755,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="20" t="s">
-        <v>101</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="s">
-        <v>102</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1952,10 +2768,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>103</v>
+        <v>155</v>
       </c>
       <c r="C4" s="25" t="s">
-        <v>104</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1963,10 +2779,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>105</v>
+        <v>157</v>
       </c>
       <c r="C5" s="25" t="s">
-        <v>106</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1974,10 +2790,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>107</v>
+        <v>159</v>
       </c>
       <c r="C6" s="25" t="s">
-        <v>108</v>
+        <v>160</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1985,10 +2801,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>109</v>
+        <v>161</v>
       </c>
       <c r="C7" s="25" t="s">
-        <v>110</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1996,10 +2812,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>111</v>
+        <v>163</v>
       </c>
       <c r="C8" s="25" t="s">
-        <v>112</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2007,15 +2823,15 @@
         <v>6</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>113</v>
+        <v>165</v>
       </c>
       <c r="C9" s="25" t="s">
-        <v>114</v>
+        <v>166</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="s">
-        <v>115</v>
+        <v>167</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2023,22 +2839,22 @@
         <v>2</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>116</v>
+        <v>168</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>117</v>
+        <v>169</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>118</v>
+        <v>170</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>119</v>
+        <v>171</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>120</v>
+        <v>172</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>121</v>
+        <v>173</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2046,10 +2862,10 @@
         <v>1</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>122</v>
+        <v>174</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>123</v>
+        <v>175</v>
       </c>
       <c r="D13" s="27" t="n">
         <v>30000</v>
@@ -2071,10 +2887,10 @@
         <v>2</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>124</v>
+        <v>176</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>125</v>
+        <v>177</v>
       </c>
       <c r="D14" s="27" t="n">
         <v>75000</v>
@@ -2096,10 +2912,10 @@
         <v>3</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>126</v>
+        <v>178</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>127</v>
+        <v>179</v>
       </c>
       <c r="D15" s="27" t="n">
         <v>75000</v>
@@ -2121,10 +2937,10 @@
         <v>4</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>128</v>
+        <v>180</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>129</v>
+        <v>181</v>
       </c>
       <c r="D16" s="27" t="n">
         <v>40000</v>
@@ -2146,10 +2962,10 @@
         <v>5</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>130</v>
+        <v>182</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>131</v>
+        <v>183</v>
       </c>
       <c r="D17" s="27" t="n">
         <v>110000</v>
@@ -2171,10 +2987,10 @@
         <v>6</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>132</v>
+        <v>184</v>
       </c>
       <c r="C18" s="26" t="s">
-        <v>133</v>
+        <v>185</v>
       </c>
       <c r="D18" s="27" t="n">
         <v>80000</v>
@@ -2196,10 +3012,10 @@
         <v>7</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>134</v>
+        <v>186</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>135</v>
+        <v>187</v>
       </c>
       <c r="D19" s="27" t="n">
         <v>270000</v>
@@ -2221,10 +3037,10 @@
         <v>8</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>136</v>
+        <v>188</v>
       </c>
       <c r="C20" s="26" t="s">
-        <v>137</v>
+        <v>189</v>
       </c>
       <c r="D20" s="27" t="n">
         <v>75000</v>
@@ -2246,10 +3062,10 @@
         <v>9</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>138</v>
+        <v>190</v>
       </c>
       <c r="C21" s="26" t="s">
-        <v>139</v>
+        <v>191</v>
       </c>
       <c r="D21" s="27" t="n">
         <v>30000</v>
@@ -2269,7 +3085,7 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="29"/>
       <c r="B22" s="30" t="s">
-        <v>140</v>
+        <v>192</v>
       </c>
       <c r="C22" s="29"/>
       <c r="D22" s="31" t="n">
@@ -2291,12 +3107,12 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="22" t="s">
-        <v>141</v>
+        <v>193</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="32" t="s">
-        <v>142</v>
+        <v>194</v>
       </c>
       <c r="C25" s="33" t="n">
         <f aca="false">COUNTA(Itinerario!B6:B25)</f>
@@ -2305,7 +3121,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="32" t="s">
-        <v>143</v>
+        <v>195</v>
       </c>
       <c r="C26" s="33" t="n">
         <f aca="false">COUNTA(Itinerario!A6:A25)</f>
@@ -2314,7 +3130,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="32" t="s">
-        <v>144</v>
+        <v>196</v>
       </c>
       <c r="C27" s="33" t="n">
         <f aca="false">COUNTA(B13:B21)</f>
@@ -2323,7 +3139,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="32" t="s">
-        <v>145</v>
+        <v>197</v>
       </c>
       <c r="C28" s="33" t="n">
         <f aca="false">F22</f>
@@ -2332,7 +3148,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="32" t="s">
-        <v>146</v>
+        <v>198</v>
       </c>
       <c r="C29" s="33" t="n">
         <f aca="false">G22</f>
@@ -2341,50 +3157,50 @@
     </row>
     <row r="31" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="34" t="s">
-        <v>147</v>
+        <v>199</v>
       </c>
       <c r="C31" s="25" t="s">
-        <v>148</v>
+        <v>200</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="34" t="s">
-        <v>149</v>
+        <v>201</v>
       </c>
       <c r="C32" s="25" t="s">
-        <v>150</v>
+        <v>202</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="34" t="s">
-        <v>151</v>
+        <v>203</v>
       </c>
       <c r="C33" s="25" t="s">
-        <v>152</v>
+        <v>204</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="34" t="s">
-        <v>153</v>
+        <v>205</v>
       </c>
       <c r="C34" s="25" t="s">
-        <v>154</v>
+        <v>206</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="34" t="s">
-        <v>155</v>
+        <v>207</v>
       </c>
       <c r="C35" s="25" t="s">
-        <v>156</v>
+        <v>208</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="34" t="s">
-        <v>157</v>
+        <v>209</v>
       </c>
       <c r="C36" s="25" t="s">
-        <v>158</v>
+        <v>210</v>
       </c>
     </row>
   </sheetData>

</xml_diff>